<commit_message>
store/map.edf acc 8 banner
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralA.xlsx
+++ b/gu_in/Map.edf/neutralA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E81B0C1-CD01-4DF5-9786-7A2E9AE5B729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6233E46B-B982-4C8B-9227-05E3CF8DF5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13065" yWindow="1365" windowWidth="10110" windowHeight="11205" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2896" uniqueCount="1391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2912" uniqueCount="1407">
   <si>
     <t>char[32]</t>
   </si>
@@ -4211,6 +4211,54 @@
   </si>
   <si>
     <t>bd131B1</t>
+  </si>
+  <si>
+    <t>sd131D3</t>
+  </si>
+  <si>
+    <t>bd131D3</t>
+  </si>
+  <si>
+    <t>sd131D4</t>
+  </si>
+  <si>
+    <t>bd131D4</t>
+  </si>
+  <si>
+    <t>sd131D5</t>
+  </si>
+  <si>
+    <t>bd131D5</t>
+  </si>
+  <si>
+    <t>sd131D7</t>
+  </si>
+  <si>
+    <t>bd131D7</t>
+  </si>
+  <si>
+    <t>sd131D6</t>
+  </si>
+  <si>
+    <t>bd131D6</t>
+  </si>
+  <si>
+    <t>sd131D8</t>
+  </si>
+  <si>
+    <t>bd131D8</t>
+  </si>
+  <si>
+    <t>sd131D9</t>
+  </si>
+  <si>
+    <t>bd131D9</t>
+  </si>
+  <si>
+    <t>sd131E0</t>
+  </si>
+  <si>
+    <t>bd131E0</t>
   </si>
 </sst>
 </file>
@@ -43060,7 +43108,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H226"/>
+  <dimension ref="A1:H242"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -48936,6 +48984,422 @@
         <v>20</v>
       </c>
       <c r="H226" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8">
+      <c r="A227" s="1" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B227" s="1">
+        <v>356</v>
+      </c>
+      <c r="C227" s="1">
+        <v>-8071</v>
+      </c>
+      <c r="D227" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E227" s="1">
+        <v>-5385</v>
+      </c>
+      <c r="F227" s="1">
+        <v>20</v>
+      </c>
+      <c r="G227" s="1">
+        <v>20</v>
+      </c>
+      <c r="H227" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8">
+      <c r="A228" s="1" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B228" s="1">
+        <v>355</v>
+      </c>
+      <c r="C228" s="1">
+        <v>-8071</v>
+      </c>
+      <c r="D228" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E228" s="1">
+        <v>-5385</v>
+      </c>
+      <c r="F228" s="1">
+        <v>20</v>
+      </c>
+      <c r="G228" s="1">
+        <v>20</v>
+      </c>
+      <c r="H228" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8">
+      <c r="A229" s="1" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B229" s="1">
+        <v>356</v>
+      </c>
+      <c r="C229" s="1">
+        <v>-8005</v>
+      </c>
+      <c r="D229" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E229" s="1">
+        <v>-5390</v>
+      </c>
+      <c r="F229" s="1">
+        <v>20</v>
+      </c>
+      <c r="G229" s="1">
+        <v>20</v>
+      </c>
+      <c r="H229" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8">
+      <c r="A230" s="1" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B230" s="1">
+        <v>355</v>
+      </c>
+      <c r="C230" s="1">
+        <v>-8005</v>
+      </c>
+      <c r="D230" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E230" s="1">
+        <v>-5390</v>
+      </c>
+      <c r="F230" s="1">
+        <v>20</v>
+      </c>
+      <c r="G230" s="1">
+        <v>20</v>
+      </c>
+      <c r="H230" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8">
+      <c r="A231" s="1" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B231" s="1">
+        <v>356</v>
+      </c>
+      <c r="C231" s="1">
+        <v>-7924</v>
+      </c>
+      <c r="D231" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E231" s="1">
+        <v>-5395</v>
+      </c>
+      <c r="F231" s="1">
+        <v>20</v>
+      </c>
+      <c r="G231" s="1">
+        <v>20</v>
+      </c>
+      <c r="H231" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8">
+      <c r="A232" s="1" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B232" s="1">
+        <v>355</v>
+      </c>
+      <c r="C232" s="1">
+        <v>-7924</v>
+      </c>
+      <c r="D232" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E232" s="1">
+        <v>-5395</v>
+      </c>
+      <c r="F232" s="1">
+        <v>20</v>
+      </c>
+      <c r="G232" s="1">
+        <v>20</v>
+      </c>
+      <c r="H232" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8">
+      <c r="A233" s="1" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B233" s="1">
+        <v>356</v>
+      </c>
+      <c r="C233" s="1">
+        <v>-7831</v>
+      </c>
+      <c r="D233" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E233" s="1">
+        <v>-5401</v>
+      </c>
+      <c r="F233" s="1">
+        <v>20</v>
+      </c>
+      <c r="G233" s="1">
+        <v>20</v>
+      </c>
+      <c r="H233" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8">
+      <c r="A234" s="1" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B234" s="1">
+        <v>355</v>
+      </c>
+      <c r="C234" s="1">
+        <v>-7831</v>
+      </c>
+      <c r="D234" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E234" s="1">
+        <v>-5401</v>
+      </c>
+      <c r="F234" s="1">
+        <v>20</v>
+      </c>
+      <c r="G234" s="1">
+        <v>20</v>
+      </c>
+      <c r="H234" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8">
+      <c r="A235" s="1" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B235" s="1">
+        <v>356</v>
+      </c>
+      <c r="C235" s="1">
+        <v>-8071</v>
+      </c>
+      <c r="D235" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E235" s="1">
+        <v>-5582</v>
+      </c>
+      <c r="F235" s="1">
+        <v>20</v>
+      </c>
+      <c r="G235" s="1">
+        <v>20</v>
+      </c>
+      <c r="H235" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="236" spans="1:8">
+      <c r="A236" s="1" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B236" s="1">
+        <v>355</v>
+      </c>
+      <c r="C236" s="1">
+        <v>-8071</v>
+      </c>
+      <c r="D236" s="1">
+        <v>1037</v>
+      </c>
+      <c r="E236" s="1">
+        <v>-5582</v>
+      </c>
+      <c r="F236" s="1">
+        <v>20</v>
+      </c>
+      <c r="G236" s="1">
+        <v>20</v>
+      </c>
+      <c r="H236" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="237" spans="1:8">
+      <c r="A237" s="1" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B237" s="1">
+        <v>356</v>
+      </c>
+      <c r="C237" s="1">
+        <v>-7993</v>
+      </c>
+      <c r="D237" s="1">
+        <v>1035</v>
+      </c>
+      <c r="E237" s="1">
+        <v>-5581</v>
+      </c>
+      <c r="F237" s="1">
+        <v>20</v>
+      </c>
+      <c r="G237" s="1">
+        <v>20</v>
+      </c>
+      <c r="H237" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="238" spans="1:8">
+      <c r="A238" s="1" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B238" s="1">
+        <v>355</v>
+      </c>
+      <c r="C238" s="1">
+        <v>-7993</v>
+      </c>
+      <c r="D238" s="1">
+        <v>1035</v>
+      </c>
+      <c r="E238" s="1">
+        <v>-5581</v>
+      </c>
+      <c r="F238" s="1">
+        <v>20</v>
+      </c>
+      <c r="G238" s="1">
+        <v>20</v>
+      </c>
+      <c r="H238" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="239" spans="1:8">
+      <c r="A239" s="1" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B239" s="1">
+        <v>356</v>
+      </c>
+      <c r="C239" s="1">
+        <v>-7919</v>
+      </c>
+      <c r="D239" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E239" s="1">
+        <v>-5579</v>
+      </c>
+      <c r="F239" s="1">
+        <v>20</v>
+      </c>
+      <c r="G239" s="1">
+        <v>20</v>
+      </c>
+      <c r="H239" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="240" spans="1:8">
+      <c r="A240" s="1" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B240" s="1">
+        <v>355</v>
+      </c>
+      <c r="C240" s="1">
+        <v>-7919</v>
+      </c>
+      <c r="D240" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E240" s="1">
+        <v>-5579</v>
+      </c>
+      <c r="F240" s="1">
+        <v>20</v>
+      </c>
+      <c r="G240" s="1">
+        <v>20</v>
+      </c>
+      <c r="H240" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="241" spans="1:8">
+      <c r="A241" s="1" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B241" s="1">
+        <v>356</v>
+      </c>
+      <c r="C241" s="1">
+        <v>-7834</v>
+      </c>
+      <c r="D241" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E241" s="1">
+        <v>-5577</v>
+      </c>
+      <c r="F241" s="1">
+        <v>20</v>
+      </c>
+      <c r="G241" s="1">
+        <v>20</v>
+      </c>
+      <c r="H241" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="242" spans="1:8">
+      <c r="A242" s="1" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B242" s="1">
+        <v>355</v>
+      </c>
+      <c r="C242" s="1">
+        <v>-7834</v>
+      </c>
+      <c r="D242" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E242" s="1">
+        <v>-5577</v>
+      </c>
+      <c r="F242" s="1">
+        <v>20</v>
+      </c>
+      <c r="G242" s="1">
+        <v>20</v>
+      </c>
+      <c r="H242" s="1">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
item/map.edf bells banner 1 fix & 4 banner acc
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralA.xlsx
+++ b/gu_in/Map.edf/neutralA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6233E46B-B982-4C8B-9227-05E3CF8DF5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D4119A-0A8C-437A-AFC7-191075B88FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13065" yWindow="1365" windowWidth="10110" windowHeight="11205" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -4265,13 +4265,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4281,6 +4288,17 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="42"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -4300,14 +4318,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -48988,418 +49010,418 @@
       </c>
     </row>
     <row r="227" spans="1:8">
-      <c r="A227" s="1" t="s">
+      <c r="A227" s="3" t="s">
         <v>1391</v>
       </c>
-      <c r="B227" s="1">
+      <c r="B227" s="3">
         <v>356</v>
       </c>
-      <c r="C227" s="1">
+      <c r="C227" s="3">
+        <v>-8518</v>
+      </c>
+      <c r="D227" s="3">
+        <v>1121</v>
+      </c>
+      <c r="E227" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F227" s="3">
+        <v>20</v>
+      </c>
+      <c r="G227" s="3">
+        <v>20</v>
+      </c>
+      <c r="H227" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8">
+      <c r="A228" s="3" t="s">
+        <v>1392</v>
+      </c>
+      <c r="B228" s="3">
+        <v>355</v>
+      </c>
+      <c r="C228" s="3">
+        <v>-8518</v>
+      </c>
+      <c r="D228" s="3">
+        <v>1121</v>
+      </c>
+      <c r="E228" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F228" s="3">
+        <v>20</v>
+      </c>
+      <c r="G228" s="3">
+        <v>20</v>
+      </c>
+      <c r="H228" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8">
+      <c r="A229" s="3" t="s">
+        <v>1393</v>
+      </c>
+      <c r="B229" s="3">
+        <v>356</v>
+      </c>
+      <c r="C229" s="3">
+        <v>-8430</v>
+      </c>
+      <c r="D229" s="3">
+        <v>1101</v>
+      </c>
+      <c r="E229" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F229" s="3">
+        <v>20</v>
+      </c>
+      <c r="G229" s="3">
+        <v>20</v>
+      </c>
+      <c r="H229" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8">
+      <c r="A230" s="3" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B230" s="3">
+        <v>355</v>
+      </c>
+      <c r="C230" s="3">
+        <v>-8430</v>
+      </c>
+      <c r="D230" s="3">
+        <v>1101</v>
+      </c>
+      <c r="E230" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F230" s="3">
+        <v>20</v>
+      </c>
+      <c r="G230" s="3">
+        <v>20</v>
+      </c>
+      <c r="H230" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8">
+      <c r="A231" s="3" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B231" s="3">
+        <v>356</v>
+      </c>
+      <c r="C231" s="3">
+        <v>-8342</v>
+      </c>
+      <c r="D231" s="3">
+        <v>1082</v>
+      </c>
+      <c r="E231" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F231" s="3">
+        <v>20</v>
+      </c>
+      <c r="G231" s="3">
+        <v>20</v>
+      </c>
+      <c r="H231" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8">
+      <c r="A232" s="3" t="s">
+        <v>1396</v>
+      </c>
+      <c r="B232" s="3">
+        <v>355</v>
+      </c>
+      <c r="C232" s="3">
+        <v>-8342</v>
+      </c>
+      <c r="D232" s="3">
+        <v>1082</v>
+      </c>
+      <c r="E232" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F232" s="3">
+        <v>20</v>
+      </c>
+      <c r="G232" s="3">
+        <v>20</v>
+      </c>
+      <c r="H232" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8">
+      <c r="A233" s="3" t="s">
+        <v>1399</v>
+      </c>
+      <c r="B233" s="3">
+        <v>356</v>
+      </c>
+      <c r="C233" s="3">
+        <v>-8254</v>
+      </c>
+      <c r="D233" s="3">
+        <v>1062</v>
+      </c>
+      <c r="E233" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F233" s="3">
+        <v>20</v>
+      </c>
+      <c r="G233" s="3">
+        <v>20</v>
+      </c>
+      <c r="H233" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="234" spans="1:8">
+      <c r="A234" s="3" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B234" s="3">
+        <v>355</v>
+      </c>
+      <c r="C234" s="3">
+        <v>-8254</v>
+      </c>
+      <c r="D234" s="3">
+        <v>1062</v>
+      </c>
+      <c r="E234" s="3">
+        <v>-5402</v>
+      </c>
+      <c r="F234" s="3">
+        <v>20</v>
+      </c>
+      <c r="G234" s="3">
+        <v>20</v>
+      </c>
+      <c r="H234" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="235" spans="1:8">
+      <c r="A235" s="2" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B235" s="2">
+        <v>356</v>
+      </c>
+      <c r="C235" s="2">
         <v>-8071</v>
       </c>
-      <c r="D227" s="1">
+      <c r="D235" s="2">
         <v>1037</v>
       </c>
-      <c r="E227" s="1">
-        <v>-5385</v>
-      </c>
-      <c r="F227" s="1">
+      <c r="E235" s="2">
+        <v>-5582</v>
+      </c>
+      <c r="F235" s="2">
         <v>20</v>
       </c>
-      <c r="G227" s="1">
+      <c r="G235" s="2">
         <v>20</v>
       </c>
-      <c r="H227" s="1">
+      <c r="H235" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="228" spans="1:8">
-      <c r="A228" s="1" t="s">
-        <v>1392</v>
-      </c>
-      <c r="B228" s="1">
+    <row r="236" spans="1:8">
+      <c r="A236" s="2" t="s">
+        <v>1398</v>
+      </c>
+      <c r="B236" s="2">
         <v>355</v>
       </c>
-      <c r="C228" s="1">
+      <c r="C236" s="2">
         <v>-8071</v>
       </c>
-      <c r="D228" s="1">
+      <c r="D236" s="2">
         <v>1037</v>
       </c>
-      <c r="E228" s="1">
-        <v>-5385</v>
-      </c>
-      <c r="F228" s="1">
+      <c r="E236" s="2">
+        <v>-5582</v>
+      </c>
+      <c r="F236" s="2">
         <v>20</v>
       </c>
-      <c r="G228" s="1">
+      <c r="G236" s="2">
         <v>20</v>
       </c>
-      <c r="H228" s="1">
+      <c r="H236" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="229" spans="1:8">
-      <c r="A229" s="1" t="s">
-        <v>1393</v>
-      </c>
-      <c r="B229" s="1">
+    <row r="237" spans="1:8">
+      <c r="A237" s="2" t="s">
+        <v>1401</v>
+      </c>
+      <c r="B237" s="2">
         <v>356</v>
       </c>
-      <c r="C229" s="1">
-        <v>-8005</v>
-      </c>
-      <c r="D229" s="1">
-        <v>1037</v>
-      </c>
-      <c r="E229" s="1">
-        <v>-5390</v>
-      </c>
-      <c r="F229" s="1">
+      <c r="C237" s="2">
+        <v>-7993</v>
+      </c>
+      <c r="D237" s="2">
+        <v>1035</v>
+      </c>
+      <c r="E237" s="2">
+        <v>-5581</v>
+      </c>
+      <c r="F237" s="2">
         <v>20</v>
       </c>
-      <c r="G229" s="1">
+      <c r="G237" s="2">
         <v>20</v>
       </c>
-      <c r="H229" s="1">
+      <c r="H237" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="230" spans="1:8">
-      <c r="A230" s="1" t="s">
-        <v>1394</v>
-      </c>
-      <c r="B230" s="1">
+    <row r="238" spans="1:8">
+      <c r="A238" s="2" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B238" s="2">
         <v>355</v>
       </c>
-      <c r="C230" s="1">
-        <v>-8005</v>
-      </c>
-      <c r="D230" s="1">
-        <v>1037</v>
-      </c>
-      <c r="E230" s="1">
-        <v>-5390</v>
-      </c>
-      <c r="F230" s="1">
+      <c r="C238" s="2">
+        <v>-7993</v>
+      </c>
+      <c r="D238" s="2">
+        <v>1035</v>
+      </c>
+      <c r="E238" s="2">
+        <v>-5581</v>
+      </c>
+      <c r="F238" s="2">
         <v>20</v>
       </c>
-      <c r="G230" s="1">
+      <c r="G238" s="2">
         <v>20</v>
       </c>
-      <c r="H230" s="1">
+      <c r="H238" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="231" spans="1:8">
-      <c r="A231" s="1" t="s">
-        <v>1395</v>
-      </c>
-      <c r="B231" s="1">
+    <row r="239" spans="1:8">
+      <c r="A239" s="2" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B239" s="2">
         <v>356</v>
       </c>
-      <c r="C231" s="1">
-        <v>-7924</v>
-      </c>
-      <c r="D231" s="1">
+      <c r="C239" s="2">
+        <v>-7919</v>
+      </c>
+      <c r="D239" s="2">
         <v>1034</v>
       </c>
-      <c r="E231" s="1">
-        <v>-5395</v>
-      </c>
-      <c r="F231" s="1">
+      <c r="E239" s="2">
+        <v>-5579</v>
+      </c>
+      <c r="F239" s="2">
         <v>20</v>
       </c>
-      <c r="G231" s="1">
+      <c r="G239" s="2">
         <v>20</v>
       </c>
-      <c r="H231" s="1">
+      <c r="H239" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="232" spans="1:8">
-      <c r="A232" s="1" t="s">
-        <v>1396</v>
-      </c>
-      <c r="B232" s="1">
+    <row r="240" spans="1:8">
+      <c r="A240" s="2" t="s">
+        <v>1404</v>
+      </c>
+      <c r="B240" s="2">
         <v>355</v>
       </c>
-      <c r="C232" s="1">
-        <v>-7924</v>
-      </c>
-      <c r="D232" s="1">
+      <c r="C240" s="2">
+        <v>-7919</v>
+      </c>
+      <c r="D240" s="2">
         <v>1034</v>
       </c>
-      <c r="E232" s="1">
-        <v>-5395</v>
-      </c>
-      <c r="F232" s="1">
+      <c r="E240" s="2">
+        <v>-5579</v>
+      </c>
+      <c r="F240" s="2">
         <v>20</v>
       </c>
-      <c r="G232" s="1">
+      <c r="G240" s="2">
         <v>20</v>
       </c>
-      <c r="H232" s="1">
+      <c r="H240" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="233" spans="1:8">
-      <c r="A233" s="1" t="s">
-        <v>1399</v>
-      </c>
-      <c r="B233" s="1">
+    <row r="241" spans="1:8">
+      <c r="A241" s="2" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B241" s="2">
         <v>356</v>
       </c>
-      <c r="C233" s="1">
-        <v>-7831</v>
-      </c>
-      <c r="D233" s="1">
+      <c r="C241" s="2">
+        <v>-7834</v>
+      </c>
+      <c r="D241" s="2">
         <v>1034</v>
       </c>
-      <c r="E233" s="1">
-        <v>-5401</v>
-      </c>
-      <c r="F233" s="1">
+      <c r="E241" s="2">
+        <v>-5577</v>
+      </c>
+      <c r="F241" s="2">
         <v>20</v>
       </c>
-      <c r="G233" s="1">
+      <c r="G241" s="2">
         <v>20</v>
       </c>
-      <c r="H233" s="1">
+      <c r="H241" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="234" spans="1:8">
-      <c r="A234" s="1" t="s">
-        <v>1400</v>
-      </c>
-      <c r="B234" s="1">
+    <row r="242" spans="1:8">
+      <c r="A242" s="2" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B242" s="2">
         <v>355</v>
       </c>
-      <c r="C234" s="1">
-        <v>-7831</v>
-      </c>
-      <c r="D234" s="1">
+      <c r="C242" s="2">
+        <v>-7834</v>
+      </c>
+      <c r="D242" s="2">
         <v>1034</v>
       </c>
-      <c r="E234" s="1">
-        <v>-5401</v>
-      </c>
-      <c r="F234" s="1">
+      <c r="E242" s="2">
+        <v>-5577</v>
+      </c>
+      <c r="F242" s="2">
         <v>20</v>
       </c>
-      <c r="G234" s="1">
+      <c r="G242" s="2">
         <v>20</v>
       </c>
-      <c r="H234" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="235" spans="1:8">
-      <c r="A235" s="1" t="s">
-        <v>1397</v>
-      </c>
-      <c r="B235" s="1">
-        <v>356</v>
-      </c>
-      <c r="C235" s="1">
-        <v>-8071</v>
-      </c>
-      <c r="D235" s="1">
-        <v>1037</v>
-      </c>
-      <c r="E235" s="1">
-        <v>-5582</v>
-      </c>
-      <c r="F235" s="1">
-        <v>20</v>
-      </c>
-      <c r="G235" s="1">
-        <v>20</v>
-      </c>
-      <c r="H235" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="236" spans="1:8">
-      <c r="A236" s="1" t="s">
-        <v>1398</v>
-      </c>
-      <c r="B236" s="1">
-        <v>355</v>
-      </c>
-      <c r="C236" s="1">
-        <v>-8071</v>
-      </c>
-      <c r="D236" s="1">
-        <v>1037</v>
-      </c>
-      <c r="E236" s="1">
-        <v>-5582</v>
-      </c>
-      <c r="F236" s="1">
-        <v>20</v>
-      </c>
-      <c r="G236" s="1">
-        <v>20</v>
-      </c>
-      <c r="H236" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="237" spans="1:8">
-      <c r="A237" s="1" t="s">
-        <v>1401</v>
-      </c>
-      <c r="B237" s="1">
-        <v>356</v>
-      </c>
-      <c r="C237" s="1">
-        <v>-7993</v>
-      </c>
-      <c r="D237" s="1">
-        <v>1035</v>
-      </c>
-      <c r="E237" s="1">
-        <v>-5581</v>
-      </c>
-      <c r="F237" s="1">
-        <v>20</v>
-      </c>
-      <c r="G237" s="1">
-        <v>20</v>
-      </c>
-      <c r="H237" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="238" spans="1:8">
-      <c r="A238" s="1" t="s">
-        <v>1402</v>
-      </c>
-      <c r="B238" s="1">
-        <v>355</v>
-      </c>
-      <c r="C238" s="1">
-        <v>-7993</v>
-      </c>
-      <c r="D238" s="1">
-        <v>1035</v>
-      </c>
-      <c r="E238" s="1">
-        <v>-5581</v>
-      </c>
-      <c r="F238" s="1">
-        <v>20</v>
-      </c>
-      <c r="G238" s="1">
-        <v>20</v>
-      </c>
-      <c r="H238" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="239" spans="1:8">
-      <c r="A239" s="1" t="s">
-        <v>1403</v>
-      </c>
-      <c r="B239" s="1">
-        <v>356</v>
-      </c>
-      <c r="C239" s="1">
-        <v>-7919</v>
-      </c>
-      <c r="D239" s="1">
-        <v>1034</v>
-      </c>
-      <c r="E239" s="1">
-        <v>-5579</v>
-      </c>
-      <c r="F239" s="1">
-        <v>20</v>
-      </c>
-      <c r="G239" s="1">
-        <v>20</v>
-      </c>
-      <c r="H239" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="240" spans="1:8">
-      <c r="A240" s="1" t="s">
-        <v>1404</v>
-      </c>
-      <c r="B240" s="1">
-        <v>355</v>
-      </c>
-      <c r="C240" s="1">
-        <v>-7919</v>
-      </c>
-      <c r="D240" s="1">
-        <v>1034</v>
-      </c>
-      <c r="E240" s="1">
-        <v>-5579</v>
-      </c>
-      <c r="F240" s="1">
-        <v>20</v>
-      </c>
-      <c r="G240" s="1">
-        <v>20</v>
-      </c>
-      <c r="H240" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="241" spans="1:8">
-      <c r="A241" s="1" t="s">
-        <v>1405</v>
-      </c>
-      <c r="B241" s="1">
-        <v>356</v>
-      </c>
-      <c r="C241" s="1">
-        <v>-7834</v>
-      </c>
-      <c r="D241" s="1">
-        <v>1034</v>
-      </c>
-      <c r="E241" s="1">
-        <v>-5577</v>
-      </c>
-      <c r="F241" s="1">
-        <v>20</v>
-      </c>
-      <c r="G241" s="1">
-        <v>20</v>
-      </c>
-      <c r="H241" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="242" spans="1:8">
-      <c r="A242" s="1" t="s">
-        <v>1406</v>
-      </c>
-      <c r="B242" s="1">
-        <v>355</v>
-      </c>
-      <c r="C242" s="1">
-        <v>-7834</v>
-      </c>
-      <c r="D242" s="1">
-        <v>1034</v>
-      </c>
-      <c r="E242" s="1">
-        <v>-5577</v>
-      </c>
-      <c r="F242" s="1">
-        <v>20</v>
-      </c>
-      <c r="G242" s="1">
-        <v>20</v>
-      </c>
-      <c r="H242" s="1">
+      <c r="H242" s="2">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
map.edf acc banner fix
</commit_message>
<xml_diff>
--- a/gu_in/Map.edf/neutralA.xlsx
+++ b/gu_in/Map.edf/neutralA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\emay.dev\Parser_1.0.2\Database\gu_in\Map.edf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87D4119A-0A8C-437A-AFC7-191075B88FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B199A29-45A2-46F3-9066-DBF33EEB715A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4278,7 +4278,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4293,12 +4293,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -4322,10 +4316,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -49010,210 +49003,210 @@
       </c>
     </row>
     <row r="227" spans="1:8">
-      <c r="A227" s="3" t="s">
+      <c r="A227" s="2" t="s">
         <v>1391</v>
       </c>
-      <c r="B227" s="3">
+      <c r="B227" s="2">
         <v>356</v>
       </c>
-      <c r="C227" s="3">
+      <c r="C227" s="2">
         <v>-8518</v>
       </c>
-      <c r="D227" s="3">
+      <c r="D227" s="2">
         <v>1121</v>
       </c>
-      <c r="E227" s="3">
+      <c r="E227" s="2">
         <v>-5402</v>
       </c>
-      <c r="F227" s="3">
+      <c r="F227" s="2">
         <v>20</v>
       </c>
-      <c r="G227" s="3">
+      <c r="G227" s="2">
         <v>20</v>
       </c>
-      <c r="H227" s="3">
+      <c r="H227" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="228" spans="1:8">
-      <c r="A228" s="3" t="s">
+      <c r="A228" s="2" t="s">
         <v>1392</v>
       </c>
-      <c r="B228" s="3">
+      <c r="B228" s="2">
         <v>355</v>
       </c>
-      <c r="C228" s="3">
+      <c r="C228" s="2">
         <v>-8518</v>
       </c>
-      <c r="D228" s="3">
+      <c r="D228" s="2">
         <v>1121</v>
       </c>
-      <c r="E228" s="3">
+      <c r="E228" s="2">
         <v>-5402</v>
       </c>
-      <c r="F228" s="3">
+      <c r="F228" s="2">
         <v>20</v>
       </c>
-      <c r="G228" s="3">
+      <c r="G228" s="2">
         <v>20</v>
       </c>
-      <c r="H228" s="3">
+      <c r="H228" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="229" spans="1:8">
-      <c r="A229" s="3" t="s">
+      <c r="A229" s="2" t="s">
         <v>1393</v>
       </c>
-      <c r="B229" s="3">
+      <c r="B229" s="2">
         <v>356</v>
       </c>
-      <c r="C229" s="3">
+      <c r="C229" s="2">
         <v>-8430</v>
       </c>
-      <c r="D229" s="3">
+      <c r="D229" s="2">
         <v>1101</v>
       </c>
-      <c r="E229" s="3">
+      <c r="E229" s="2">
         <v>-5402</v>
       </c>
-      <c r="F229" s="3">
+      <c r="F229" s="2">
         <v>20</v>
       </c>
-      <c r="G229" s="3">
+      <c r="G229" s="2">
         <v>20</v>
       </c>
-      <c r="H229" s="3">
+      <c r="H229" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="230" spans="1:8">
-      <c r="A230" s="3" t="s">
+      <c r="A230" s="2" t="s">
         <v>1394</v>
       </c>
-      <c r="B230" s="3">
+      <c r="B230" s="2">
         <v>355</v>
       </c>
-      <c r="C230" s="3">
+      <c r="C230" s="2">
         <v>-8430</v>
       </c>
-      <c r="D230" s="3">
+      <c r="D230" s="2">
         <v>1101</v>
       </c>
-      <c r="E230" s="3">
+      <c r="E230" s="2">
         <v>-5402</v>
       </c>
-      <c r="F230" s="3">
+      <c r="F230" s="2">
         <v>20</v>
       </c>
-      <c r="G230" s="3">
+      <c r="G230" s="2">
         <v>20</v>
       </c>
-      <c r="H230" s="3">
+      <c r="H230" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="231" spans="1:8">
-      <c r="A231" s="3" t="s">
+      <c r="A231" s="2" t="s">
         <v>1395</v>
       </c>
-      <c r="B231" s="3">
+      <c r="B231" s="2">
         <v>356</v>
       </c>
-      <c r="C231" s="3">
+      <c r="C231" s="2">
         <v>-8342</v>
       </c>
-      <c r="D231" s="3">
+      <c r="D231" s="2">
         <v>1082</v>
       </c>
-      <c r="E231" s="3">
+      <c r="E231" s="2">
         <v>-5402</v>
       </c>
-      <c r="F231" s="3">
+      <c r="F231" s="2">
         <v>20</v>
       </c>
-      <c r="G231" s="3">
+      <c r="G231" s="2">
         <v>20</v>
       </c>
-      <c r="H231" s="3">
+      <c r="H231" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="232" spans="1:8">
-      <c r="A232" s="3" t="s">
+      <c r="A232" s="2" t="s">
         <v>1396</v>
       </c>
-      <c r="B232" s="3">
+      <c r="B232" s="2">
         <v>355</v>
       </c>
-      <c r="C232" s="3">
+      <c r="C232" s="2">
         <v>-8342</v>
       </c>
-      <c r="D232" s="3">
+      <c r="D232" s="2">
         <v>1082</v>
       </c>
-      <c r="E232" s="3">
+      <c r="E232" s="2">
         <v>-5402</v>
       </c>
-      <c r="F232" s="3">
+      <c r="F232" s="2">
         <v>20</v>
       </c>
-      <c r="G232" s="3">
+      <c r="G232" s="2">
         <v>20</v>
       </c>
-      <c r="H232" s="3">
+      <c r="H232" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="233" spans="1:8">
-      <c r="A233" s="3" t="s">
+      <c r="A233" s="2" t="s">
         <v>1399</v>
       </c>
-      <c r="B233" s="3">
+      <c r="B233" s="2">
         <v>356</v>
       </c>
-      <c r="C233" s="3">
+      <c r="C233" s="2">
         <v>-8254</v>
       </c>
-      <c r="D233" s="3">
+      <c r="D233" s="2">
         <v>1062</v>
       </c>
-      <c r="E233" s="3">
+      <c r="E233" s="2">
         <v>-5402</v>
       </c>
-      <c r="F233" s="3">
+      <c r="F233" s="2">
         <v>20</v>
       </c>
-      <c r="G233" s="3">
+      <c r="G233" s="2">
         <v>20</v>
       </c>
-      <c r="H233" s="3">
+      <c r="H233" s="2">
         <v>20</v>
       </c>
     </row>
     <row r="234" spans="1:8">
-      <c r="A234" s="3" t="s">
+      <c r="A234" s="2" t="s">
         <v>1400</v>
       </c>
-      <c r="B234" s="3">
+      <c r="B234" s="2">
         <v>355</v>
       </c>
-      <c r="C234" s="3">
+      <c r="C234" s="2">
         <v>-8254</v>
       </c>
-      <c r="D234" s="3">
+      <c r="D234" s="2">
         <v>1062</v>
       </c>
-      <c r="E234" s="3">
+      <c r="E234" s="2">
         <v>-5402</v>
       </c>
-      <c r="F234" s="3">
+      <c r="F234" s="2">
         <v>20</v>
       </c>
-      <c r="G234" s="3">
+      <c r="G234" s="2">
         <v>20</v>
       </c>
-      <c r="H234" s="3">
+      <c r="H234" s="2">
         <v>20</v>
       </c>
     </row>
@@ -49225,13 +49218,13 @@
         <v>356</v>
       </c>
       <c r="C235" s="2">
-        <v>-8071</v>
+        <v>-8518</v>
       </c>
       <c r="D235" s="2">
-        <v>1037</v>
+        <v>1121</v>
       </c>
       <c r="E235" s="2">
-        <v>-5582</v>
+        <v>-5565</v>
       </c>
       <c r="F235" s="2">
         <v>20</v>
@@ -49251,13 +49244,13 @@
         <v>355</v>
       </c>
       <c r="C236" s="2">
-        <v>-8071</v>
+        <v>-8518</v>
       </c>
       <c r="D236" s="2">
-        <v>1037</v>
+        <v>1121</v>
       </c>
       <c r="E236" s="2">
-        <v>-5582</v>
+        <v>-5565</v>
       </c>
       <c r="F236" s="2">
         <v>20</v>
@@ -49277,13 +49270,13 @@
         <v>356</v>
       </c>
       <c r="C237" s="2">
-        <v>-7993</v>
+        <v>-8430</v>
       </c>
       <c r="D237" s="2">
-        <v>1035</v>
+        <v>1102</v>
       </c>
       <c r="E237" s="2">
-        <v>-5581</v>
+        <v>-5565</v>
       </c>
       <c r="F237" s="2">
         <v>20</v>
@@ -49303,13 +49296,13 @@
         <v>355</v>
       </c>
       <c r="C238" s="2">
-        <v>-7993</v>
+        <v>-8430</v>
       </c>
       <c r="D238" s="2">
-        <v>1035</v>
+        <v>1102</v>
       </c>
       <c r="E238" s="2">
-        <v>-5581</v>
+        <v>-5565</v>
       </c>
       <c r="F238" s="2">
         <v>20</v>
@@ -49329,13 +49322,13 @@
         <v>356</v>
       </c>
       <c r="C239" s="2">
-        <v>-7919</v>
+        <v>-8342</v>
       </c>
       <c r="D239" s="2">
-        <v>1034</v>
+        <v>1082</v>
       </c>
       <c r="E239" s="2">
-        <v>-5579</v>
+        <v>-5565</v>
       </c>
       <c r="F239" s="2">
         <v>20</v>
@@ -49355,13 +49348,13 @@
         <v>355</v>
       </c>
       <c r="C240" s="2">
-        <v>-7919</v>
+        <v>-8342</v>
       </c>
       <c r="D240" s="2">
-        <v>1034</v>
+        <v>1082</v>
       </c>
       <c r="E240" s="2">
-        <v>-5579</v>
+        <v>-5565</v>
       </c>
       <c r="F240" s="2">
         <v>20</v>
@@ -49381,13 +49374,13 @@
         <v>356</v>
       </c>
       <c r="C241" s="2">
-        <v>-7834</v>
+        <v>-8254</v>
       </c>
       <c r="D241" s="2">
-        <v>1034</v>
+        <v>1062</v>
       </c>
       <c r="E241" s="2">
-        <v>-5577</v>
+        <v>-5566</v>
       </c>
       <c r="F241" s="2">
         <v>20</v>
@@ -49407,13 +49400,13 @@
         <v>355</v>
       </c>
       <c r="C242" s="2">
-        <v>-7834</v>
+        <v>-8254</v>
       </c>
       <c r="D242" s="2">
-        <v>1034</v>
+        <v>1062</v>
       </c>
       <c r="E242" s="2">
-        <v>-5577</v>
+        <v>-5566</v>
       </c>
       <c r="F242" s="2">
         <v>20</v>

</xml_diff>